<commit_message>
Replace sanitised sample with 15 real leads from UCI dataset (open source data)
</commit_message>
<xml_diff>
--- a/sample_output/leads_report_sample.xlsx
+++ b/sample_output/leads_report_sample.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Audit_Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -75,16 +75,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -458,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,15 +461,17 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -511,54 +507,64 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Marital</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Balance_EUR</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Housing_Loan</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Personal_Loan</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Engagement_s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Campaign_Contacts</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Prev_Outcome</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>RM_Assigned</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Last_Updated</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SAMPLE-001</t>
+          <t>LEAD-0018</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -582,46 +588,56 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>45248</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
+      <c r="K2" s="2" t="n">
         <v>1623</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="L2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>RM_Priya</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SAMPLE-002</t>
+          <t>LEAD-0658</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -645,46 +661,56 @@
           <t>tertiary</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>11008</v>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n">
-        <v>1521</v>
-      </c>
       <c r="K3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
+        <v>1540</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>RM_Arjun</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SAMPLE-003</t>
+          <t>LEAD-0384</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -708,46 +734,56 @@
           <t>tertiary</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>married</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>13853</v>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="K4" s="3" t="n">
         <v>1329</v>
       </c>
-      <c r="K4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>RM_Sofia</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>SAMPLE-004</t>
+          <t>LEAD-0462</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -771,46 +807,56 @@
           <t>tertiary</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n">
         <v>12956</v>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>940</v>
       </c>
-      <c r="K5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>RM_Marcus</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>SAMPLE-005</t>
+          <t>LEAD-0354</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -834,44 +880,784 @@
           <t>tertiary</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>divorced</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>14481</v>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="K6" s="3" t="n">
+        <v>1269</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>RM_Chen</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-1647</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>6840</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="J6" s="3" t="n">
-        <v>1269</v>
-      </c>
-      <c r="K6" s="3" t="n">
+      <c r="K7" s="3" t="n">
+        <v>1560</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>RM_Priya</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-1508</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>married</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>7192</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>1486</v>
+      </c>
+      <c r="L8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>RM_Arjun</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0396</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>13711</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>1532</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>RM_Sofia</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0190</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>married</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>19797</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>966</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>RM_Marcus</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-2433</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>5389</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>1456</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>RM_Chen</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-2371</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>divorced</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>5475</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>1032</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>RM_Priya</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-4292</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>3646</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>1710</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>RM_Arjun</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-4598</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>3445</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>1662</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>RM_Sofia</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-2735</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>divorced</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>5037</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>1437</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>RM_Marcus</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0718</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>tertiary</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>married</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>10576</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>1224</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>RM_Chen</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -882,15 +1668,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="75" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="5" max="5"/>
+    <col width="75" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -926,162 +1712,482 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>SAMPLE-001</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LEAD-0018</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>RM_Priya</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Strong candidate given a €45,248 balance and a 1,623-second prior call indicating sustained interest in financial planning.</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Following your recent detailed conversation with us, I wanted to reach out about term deposit options that could put your savings to work immediately.</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>A fixed-rate term deposit would lock in a competitive return on the €45,248 sitting in your account — with no market risk.</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>This customer is a strong wealth product candidate given their Tier A profile review, a solid €45,248 average annual balance, and highly engaged 1623-second prior call.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>"Following your recent 1623-second conversation with us, and noticing your healthy €45,248 average annual balance, I wanted to connect regarding opportunities to enhance your financial future."</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Leveraging their existing housing loan and €45,248 average annual balance for growth strategies would be a compelling angle for this 39-year-old technician.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>SAMPLE-002</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0658</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>RM_Arjun</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Management professional with tertiary education and no existing loans — ideal profile for a first term deposit commitment.</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Given your strong professional background and the detailed conversation you had with our team recently, I wanted to share a term deposit offer tailored to your income level.</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>With no current loans and a €11,008 balance, this is an opportunity to lock in a guaranteed return before rates shift.</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>This 41-year-old management professional with tertiary education and no existing loans presents a strong opportunity to optimize their wealth, especially given their current average annual balance of €11,008.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Following your recent engagement of over 1500 seconds, I wanted to connect regarding opportunities to enhance your financial growth and make the most of your income as a management professional.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>We should focus on leveraging your strong professional background to significantly grow your average annual balance of €11,008 through strategic wealth management solutions.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>SAMPLE-003</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0384</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>RM_Sofia</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>44-year-old management professional with 1,329 seconds of call engagement — clearly evaluating financial options actively.</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>You spent over 22 minutes speaking with our team recently, which tells me you are actively thinking about your financial future — I have something specific to share.</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>A 12-month term deposit at the current rate would give you a guaranteed return while you decide on longer-term strategy.</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>This 44-year-old customer in management with tertiary education, identified as a strong candidate based on profile review, demonstrated significant engagement with 1329 seconds on their last call, indicating readiness to discuss wealth opportunities.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Hello, I noticed your recent call engagement was over 1300 seconds, and I wanted to follow up specifically on how we can help you develop a robust financial strategy as you approach your peak earning years.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Despite your current average balance of €13,853, your profile as a 44-year-old married professional in management with a housing loan presents a prime opportunity to strategically grow your wealth for long-term goals.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>SAMPLE-004</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0462</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>RM_Marcus</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Previous campaign success and 940 seconds of engagement make this 28-year-old management professional a warm re-contact.</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>You subscribed to one of our products before, so you already know the value — I wanted to follow up on a new term deposit offer that builds on that.</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Given the previous successful outcome and your early career stage, a rolling short-term deposit strategy could be a strong fit.</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>This 28-year-old in management, with tertiary education, represents a strong candidate due to a previous campaign success and demonstrated high interest with 940 seconds on their last call.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Given your previous successful campaign outcome and the 940 seconds spent discussing your finances last time, I wanted to share some insights on how we can build on that momentum.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Let's discuss how to strategically grow your current assets, leveraging your management position and the insights from our previous successful engagement, to achieve your long-term financial aspirations.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>SAMPLE-005</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0354</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>RM_Chen</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior management professional, 46, with a 1,269-second call — high engagement from someone at peak earning stage.</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Following your recent conversation with us, I wanted to discuss how a term deposit could complement your current financial position as you approach your highest-earning years.</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Locking in a competitive rate now, before any potential rate changes, is particularly relevant for someone at your career stage with a €14,481 balance to grow.</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Their management position, age 46, and recent 1269-second call engagement, coupled with a profile review indicating potential for financial re-evaluation post-divorce, make them a strong wealth candidate.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Following up on your recent detailed conversation with us, I wanted to reach out and offer a brief financial check-in to ensure your current planning aligns with your goals.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Considering your management position and the need to re-evaluate financial strategies post-divorce, we can help optimize growth beyond your current €14,481 average annual balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-1647</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>RM_Priya</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>This 26-year-old in a management role with tertiary education is a strong wealth product candidate due to their existing housing loan, indicating financial responsibility, and a significant 1560-second recent call engagement suggesting high interest in financial discussions.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Building on our recent 1560-second discussion, I wanted to briefly share some insights on maximizing your financial potential at 26 years old.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Given your management role and existing housing loan at 26, the most compelling angle is to discuss long-term investment strategies to leverage your early start and maximize wealth accumulation over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-1508</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>RM_Arjun</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>This 52-year-old manager, debt-free and with tertiary education, engaged for 1486 seconds on the last call, suggesting a high readiness to explore wealth solutions despite a current average balance of €7,192.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Following your recent 1486-second engagement, I wanted to reach out regarding our wealth management solutions that align with your financial goals at 52.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Highlight how their management role and absence of a housing loan provide an excellent foundation to significantly grow or consolidate assets beyond their current €7,192 average balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0396</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>RM_Sofia</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>This customer, aged 31 with tertiary education and a Housing Loan, presents a strong long-term wealth building opportunity, further supported by a Tier B profile analysis and an impressive 1532 seconds of recent call engagement.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Following your recent detailed conversation with us, I wanted to connect regarding how we can help you effectively grow your current savings and future financial position.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Discuss strategies to enhance their existing €13,711 average annual balance, leveraging their demonstrated long-term financial commitment from their housing loan to begin significant wealth accumulation at 31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0190</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>RM_Marcus</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>This 52-year-old management professional with tertiary education and a high recent call engagement of 966 seconds, combined with a Tier B profile review, represents an excellent opportunity to explore wealth solutions beyond their current €19,797 average annual balance.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>As your RM, Marcus, I wanted to briefly connect to discuss strategies for optimizing your financial outlook, especially as you approach 52.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Emphasize how their management profession and tertiary education make them well-suited to discuss investment strategies for long-term growth and retirement planning, particularly given their current €19,797 average annual balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-2433</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>RM_Chen</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>This 30-year-old in management with tertiary education presents strong long-term growth potential and demonstrated high interest with 1456 seconds of recent call engagement, despite a modest €5,389 average annual balance, which presents a clear opportunity for wealth building.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Following our last detailed discussion that lasted over 1400 seconds, I wanted to connect regarding strategies to maximize your financial growth at this key stage of your management career.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Given your current average annual balance of €5,389 and no existing loans, the most compelling discussion will focus on establishing an early, tailored investment plan to leverage your strong earning potential and compound wealth effectively over the next few decades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-2371</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>RM_Priya</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>This 54-year-old management professional is a strong candidate given their tertiary education, previous campaign success, and significant 1032-second engagement on their last call, all while having no existing housing or personal loans.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>"Following your successful outcome from our previous campaign, I wanted to connect regarding opportunities to optimize your financial planning, particularly as you approach your pre-retirement years."</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Given your age of 54 and management background, we see an opportunity to grow your assets beyond your current €5,475 average balance, leveraging your unburdened financial position without housing or personal loans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-4292</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>RM_Arjun</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>This 38-year-old customer in management with tertiary education presents strong potential for wealth accumulation, further supported by a Tier B analysis and their recent 1710-second call engagement.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Following our recent 1710-second conversation, I wanted to connect regarding your financial growth and explore options tailored to your management career and tertiary education.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>The most compelling angle is to explore strategies for long-term wealth building, leveraging their stable management income and existing housing loan to optimize their overall financial portfolio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-4598</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>RM_Sofia</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>This 42-year-old manager with tertiary education and no existing loans presents strong untapped wealth potential, indicated by a B-tier profile analysis and a significant 1662 seconds of recent call engagement despite a modest €3,445 average annual balance.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Following up on your recent 1662-second call, I wanted to explore how we can align your financial strategy with your career stage and goals.</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Given your management position and lack of housing or personal loans, we should focus on investment opportunities to significantly grow your capital beyond your current €3,445 average annual balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-2735</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>RM_Marcus</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>This 58-year-old management professional with tertiary education is a strong wealth product candidate given their B-tier profile review and highly engaged 1437-second recent call, suggesting a readiness to discuss future financial planning despite a current average annual balance of €5,037.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>"Given your recent 1437-second call engagement, I wanted to follow up and explore opportunities to enhance your financial planning, particularly as you are 58 years old and in a management role."</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Focus on comprehensive retirement planning and leveraging their housing loan asset, exploring how funds beyond their €5,037 average annual balance can be better optimized as they approach retirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>LEAD-0718</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>RM_Chen</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>This 29-year-old management professional, with tertiary education and a robust 1224-second engagement on their last call, shows significant potential for wealth growth given their long-term horizon and current lack of housing or personal loans, highlighted by a strong profile analysis.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Building on your recent 1224-second engagement, I'd like to explore how we can align your financial strategy with your career trajectory in management.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>We should focus on establishing a strategic long-term wealth accumulation plan, leveraging their management career and current lack of housing or personal loans to maximize early investment opportunities.</t>
         </is>
       </c>
     </row>
@@ -1101,7 +2207,7 @@
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1122,19 +2228,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>2026-05-11 09:00:00</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11 01:36:22</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>LEADS_EXPORTED</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>5 sample leads exported — Week 19, 2026 (SAMPLE DATA)</t>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>15-lead sample export from UCI Bank Marketing dataset — Week 19, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>